<commit_message>
data(eval): refresh evaluation artifacts for v0.9.1
* 43-question benchmark (EU set added) -> retrieval_questions / retrieval_results
* Task 4 before/after, ablation and optimized run re-measured after the
  investment-screening lexicon fix (full: P@5 0.800 / R@10 0.925)
* Task 3 baseline report, Task 5-7 outputs and evaluation_report.md regenerated
</commit_message>
<xml_diff>
--- a/data/evaluation/entity_accuracy.xlsx
+++ b/data/evaluation/entity_accuracy.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Entity Detail'!$A$1:$F$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Entity Detail'!$A$1:$F$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -842,7 +842,7 @@
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>BIS_002; BIS_001; CASE_009; MOFCOM_002; MOFCOM_001; NIO_001; XPEV_001; DHS_001; EU_003; IRS_001</t>
+          <t>BIS_002; BIS_001; MOFCOM_002; CASE_009; MOFCOM_001; NIO_001; XPEV_001; DHS_001; EU_003; IRS_001</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1366,7 @@
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; CASE_003; TRD_002; DHS_001; WH_002; CASE_002; CASE_010; IRS_001; SNE_001</t>
+          <t>TRD_001; TRD_003; CASE_003; DHS_001; TRD_002; WH_002; CASE_002; CASE_010; IRS_001; SNE_001</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>BIS_001; BIS_002; CASE_009; DHS_001; EU_001; XPEV_001; NIO_001; IRS_001; UST_001; EU_003</t>
+          <t>BIS_001; BIS_002; CASE_009; DHS_001; EU_001; XPEV_001; NIO_001; IRS_001; MOFCOM_002; UST_001</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
       <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>TSLA_001; EU_003; UST_001; DHS_001; SNE_001; IRS_001; TRD_001; WTO_003; CASE_002; EU_001</t>
+          <t>TSLA_001; EU_003; UST_001; DHS_001; SNE_001; TRD_001; IRS_001; WTO_003; CASE_002; EU_001</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2310,7 @@
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>USMCA_001; DHS_001; CSIS_001; SNE_001; IRS_001; EU_003; UST_001; CASE_002; WTO_003; EU_001</t>
+          <t>USMCA_001; DHS_001; CSIS_001; SNE_001; IRS_001; EU_003; UST_001; TRD_001; CASE_002; WTO_003</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2418,7 @@
       <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>WTO_004; DHS_001; IRS_001; EU_001; SNE_001; WTO_002; EU_003; MOFCOM_002; TSLA_001; EU_002</t>
+          <t>WTO_004; DHS_001; IRS_001; EU_001; SNE_001; WTO_002; EU_003; MOFCOM_002; TSLA_001; TRD_001</t>
         </is>
       </c>
     </row>
@@ -2500,13 +2500,13 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="F39" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -2521,16 +2521,12 @@
         <v>2</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="M39" s="2" t="inlineStr">
-        <is>
-          <t>CASE_008</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="M39" s="2" t="inlineStr"/>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>DHS_001; IRS_001; EU_001; SNE_001; TSLA_001; EU_002; CASE_002; BIS_001; CASE_008; USMCA_001</t>
+          <t>DHS_001; IRS_001; EU_001; SNE_001; TSLA_001; MOFCOM_002; EU_002; CASE_002; BIS_001; TRD_001</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2582,7 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>SNE_001; DHS_001; EU_003; IRS_001; EU_001; IEA_001; CASE_002; UST_001; MOFCOM_002; EU_002</t>
+          <t>SNE_001; TRD_001; DHS_001; EU_003; IRS_001; EU_001; IEA_001; CASE_002; UST_001; MOFCOM_002</t>
         </is>
       </c>
     </row>
@@ -2643,6 +2639,170 @@
       <c r="N41" s="2" t="inlineStr">
         <is>
           <t>USMCA_001; WB_001; IRS_001; WTO_004; CASE_002; DHS_001; EU_001; EU_002; EU_003; TRD_001</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Q041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Market Access</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>market_access</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>我们准备向欧盟出口 EV 电池。欧盟电池法规对进入欧盟市场的电池提出了哪些强制合规要求（碳足迹、再生材料含量、供应链尽职调查、电池护照）？</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>EU; EV Battery</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K42" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L42" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>CSIS_001; UST_001</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>EU_001; DHS_001; EU_003; CSIS_001; SNE_001; IRS_001; IEA_001; UST_001; TRD_001; MOFCOM_002</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>tariff</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>欧盟对中国产纯电动车征收的最终反补贴税税率是多少？不同企业（比亚迪/吉利/上汽/特斯拉）的税率差异如何？</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>AD/CVD; China; EU; EV Battery</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K43" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L43" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>UST_001</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>EU_003; CASE_002; DHS_001; TRD_001; SNE_001; IRS_001; IEA_001; EU_001; UST_001; EU_002</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Q043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>investment_policy</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>如果中国电池企业要在欧盟建厂或收购当地电池资产，欧盟层面的外资安全审查框架和关键原材料法案会带来哪些约束（审查范围、本土化与单一第三国依赖目标）？</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>China; EU; EV Battery</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K44" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L44" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>EU_002; EU_004; DHS_001; EU_001; EU_003; CASE_002; IRS_001; SNE_001; TRD_001; MOFCOM_002</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3028,7 +3188,7 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -3056,7 +3216,7 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -3088,7 +3248,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>BIS_002; BIS_001; CASE_009; MOFCOM_002; NIO_001; XPEV_001</t>
+          <t>BIS_002; BIS_001; MOFCOM_002; CASE_009; NIO_001; XPEV_001</t>
         </is>
       </c>
     </row>
@@ -3588,11 +3748,11 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>DHS_001; CASE_002; IRS_001; SNE_001</t>
+          <t>TRD_001; DHS_001; CASE_002; IRS_001; SNE_001</t>
         </is>
       </c>
     </row>
@@ -3676,7 +3836,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>TRD_001; CASE_003; TRD_002; DHS_001; WH_002; CASE_002</t>
+          <t>TRD_001; CASE_003; DHS_001; TRD_002; WH_002; CASE_002</t>
         </is>
       </c>
     </row>
@@ -4012,7 +4172,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>DHS_001; EU_001; IRS_001; EU_003</t>
+          <t>DHS_001; EU_001; IRS_001; MOFCOM_002</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4788,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>EU_003; SNE_001; IRS_001; TRD_001; CASE_002</t>
+          <t>EU_003; SNE_001; TRD_001; IRS_001; CASE_002</t>
         </is>
       </c>
     </row>
@@ -4656,7 +4816,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>TSLA_001; EU_003; DHS_001; SNE_001; IRS_001; CASE_002</t>
+          <t>TSLA_001; EU_003; DHS_001; SNE_001; TRD_001; IRS_001</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4928,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>USMCA_001; SNE_001; IRS_001; EU_003; CASE_002</t>
+          <t>USMCA_001; SNE_001; IRS_001; EU_003; TRD_001; CASE_002</t>
         </is>
       </c>
     </row>
@@ -4796,7 +4956,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>USMCA_001; DHS_001; SNE_001; IRS_001; EU_003; CASE_002</t>
+          <t>USMCA_001; DHS_001; SNE_001; IRS_001; EU_003; TRD_001</t>
         </is>
       </c>
     </row>
@@ -5132,7 +5292,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>DHS_001; IRS_001; EU_001; SNE_001; TSLA_001; EU_002</t>
+          <t>DHS_001; IRS_001; EU_001; SNE_001; TSLA_001; MOFCOM_002</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5320,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>DHS_001; IRS_001; TSLA_001; CASE_002; BIS_001; USMCA_001</t>
+          <t>DHS_001; IRS_001; TSLA_001; MOFCOM_002; CASE_002; BIS_001</t>
         </is>
       </c>
     </row>
@@ -5188,7 +5348,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>SNE_001; EU_003; IRS_001; CASE_002; MOFCOM_002; EU_002</t>
+          <t>SNE_001; TRD_001; EU_003; IRS_001; CASE_002; MOFCOM_002</t>
         </is>
       </c>
     </row>
@@ -5216,7 +5376,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>SNE_001; DHS_001; EU_003; IRS_001; EU_001; IEA_001</t>
+          <t>SNE_001; TRD_001; DHS_001; EU_003; IRS_001; EU_001</t>
         </is>
       </c>
     </row>
@@ -5332,8 +5492,260 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Q041</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>EU_001; EU_003</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Q041</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>EV Battery</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" t="n">
+        <v>1</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>EU_001; DHS_001; EU_003; SNE_001; IRS_001; IEA_001</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>AD/CVD</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>EU_003; CASE_002</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>1</v>
+      </c>
+      <c r="E99" t="n">
+        <v>1</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>EU_003; CASE_002; TRD_001; SNE_001; IRS_001; EU_002</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" t="n">
+        <v>1</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>EU_003; EU_001; EU_002</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>EV Battery</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>1</v>
+      </c>
+      <c r="E101" t="n">
+        <v>1</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>EU_003; CASE_002; DHS_001; TRD_001; SNE_001; IRS_001</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Q043</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>EU_002; EU_003; CASE_002; IRS_001; SNE_001; TRD_001</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Q043</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" t="n">
+        <v>1</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>EU_002; EU_004; EU_001; EU_003</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Q043</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>EV Battery</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" t="n">
+        <v>1</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>EU_002; DHS_001; EU_001; EU_003; CASE_002; IRS_001</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F95"/>
+  <autoFilter ref="A1:F104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5376,11 +5788,11 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0.93</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>mean over 33 entity-bearing questions</t>
+          <t>mean over 36 entity-bearing questions</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5818,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.861</v>
+        <v>0.867</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -5421,11 +5833,11 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>of 40 (entity-free questions excluded)</t>
+          <t>of 43 (entity-free questions excluded)</t>
         </is>
       </c>
     </row>
@@ -5451,11 +5863,11 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>of 33</t>
+          <t>of 36</t>
         </is>
       </c>
     </row>
@@ -5466,11 +5878,11 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>of 33</t>
+          <t>of 36</t>
         </is>
       </c>
     </row>
@@ -5481,7 +5893,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -5533,10 +5945,10 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14">
@@ -5546,10 +5958,10 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
@@ -5559,10 +5971,10 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">

</xml_diff>